<commit_message>
Phase 3 step 3: wireless family page, model detail, selector, compare
Static pages for every published model (TR and EN), filters (OR in a group, AND across),
live count with Turkish suffixes, bottom-sheet filters on phones, compare tray, selector with
assumptions and PoE warnings, compare table with pinned label column. check:dist now fails on
any draft PID, broken internal link, End-of-Sale model in the selector, or third-party request.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/glossary.xlsx
+++ b/data/glossary.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="116">
   <si>
     <t>key</t>
   </si>
@@ -344,6 +344,21 @@
   </si>
   <si>
     <t>The date Cisco stops supporting this model.</t>
+  </si>
+  <si>
+    <t>unified</t>
+  </si>
+  <si>
+    <t>Birleşik yönetim (unified)</t>
+  </si>
+  <si>
+    <t>Unified management</t>
+  </si>
+  <si>
+    <t>Aynı model hem şirket içinde (Catalyst Center / denetleyici) hem bulutta (Meraki panosu) yönetilebilir. Bazı modellerde bunu sipariş koduna eklenen -MR eki belirler; model sayfasındaki sipariş kodlarına bakın.</t>
+  </si>
+  <si>
+    <t>The same model can be managed on-premises (Catalyst Center / controller) or in the cloud (Meraki dashboard). On some models the -MR suffix in the ordering code decides this; see the ordering codes on the model page.</t>
   </si>
 </sst>
 </file>
@@ -729,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1162,6 +1177,23 @@
         <v>110</v>
       </c>
     </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" t="s">
+        <v>113</v>
+      </c>
+      <c r="D26" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" t="s">
+        <v>115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Phase 3 step 5: review fixes (licence_required, unified, modal, compare EoS rows) and status
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/glossary.xlsx
+++ b/data/glossary.xlsx
@@ -355,10 +355,10 @@
     <t>Unified management</t>
   </si>
   <si>
-    <t>Aynı model hem şirket içinde (Catalyst Center / denetleyici) hem bulutta (Meraki panosu) yönetilebilir. Bazı modellerde bunu sipariş koduna eklenen -MR eki belirler; model sayfasındaki sipariş kodlarına bakın.</t>
-  </si>
-  <si>
-    <t>The same model can be managed on-premises (Catalyst Center / controller) or in the cloud (Meraki dashboard). On some models the -MR suffix in the ordering code decides this; see the ordering codes on the model page.</t>
+    <t>Aynı sipariş koduyla hem şirket içinde (Catalyst Center / denetleyici) hem bulutta (Meraki panosu) yönetilebilen model. Bazı modellerde bulut için ayrı bir kod (-MR eki) gerekir; onlar burada "birleşik" sayılmaz. Model sayfasındaki sipariş kodlarına bakın.</t>
+  </si>
+  <si>
+    <t>A model that can be managed on-premises (Catalyst Center / controller) or in the cloud (Meraki dashboard) under the same ordering code. Some models need a separate cloud code (the -MR suffix); those are not counted as unified here. See the ordering codes on the model page.</t>
   </si>
 </sst>
 </file>

</xml_diff>